<commit_message>
Add quarterly rate schedules to Silpo PnL calculator
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Silpo_2027_DK_Resto_Stores_PnL_Calculator.xlsx
+++ b/Silpo_2027_DK_Resto_Stores_PnL_Calculator.xlsx
@@ -11,11 +11,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L by vertical" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment &amp; partner value" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source &amp; checks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment &amp; partner value" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source &amp; checks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scenarios'!$A$5:$O$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scenarios'!$A$5:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Quarterly scenarios'!$A$6:$U$35</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -141,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -216,6 +218,12 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -780,7 +788,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Cash cost; editable</t>
+          <t>Cash activation; 6 of 12 months</t>
         </is>
       </c>
     </row>
@@ -860,7 +868,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Discount only; SF/SOF not discounted</t>
+          <t>Delivery base only; excludes SF and SOF</t>
         </is>
       </c>
     </row>
@@ -944,6 +952,26 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Historical DF campaign · DK + resto</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>14411.34</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>€ / year</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Visibility only; already included in historical demand incentives</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
@@ -1245,6 +1273,31 @@
       <c r="F29" s="8" t="inlineStr">
         <is>
           <t>% of portfolio GMV</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Eater-fee revenue (informational)</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>115473.31</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>3810.16</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="14">
+        <f>SUM(B30:D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Historical source; included in unit economics, not added again to CP</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1298,10 +1351,12 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1371,25 +1426,35 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>CP L1</t>
+          <t>CP L1 €</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>CP L2 before investments</t>
+          <t>CP L1 % GMV</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
+          <t>CP L2 €</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>CP L2 % GMV</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
           <t>Cash P&amp;L after investment</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>Cash P&amp;L % GMV</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="Q5" s="7" t="inlineStr">
         <is>
           <t>Partner saving vs baseline</t>
         </is>
@@ -1433,19 +1498,27 @@
         <f>J6-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="17">
+        <f>K6/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
         <f>K6-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M6" s="14">
-        <f>L6-($E6*Inputs!$B$7)+($F6*SUM(Inputs!$B$28:$D$28))+($G6*Inputs!$B$12)+($I6*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N6" s="17">
         <f>M6/SUM(Inputs!$B$21:$D$21)</f>
         <v/>
       </c>
-      <c r="O6" s="16">
+      <c r="O6" s="14">
+        <f>M6-(($E6*Inputs!$B$7)+($F6*SUM(Inputs!$B$28:$D$28))+($G6*Inputs!$B$12)+($I6*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P6" s="17">
+        <f>O6/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="16">
         <f>$J$6-J6</f>
         <v/>
       </c>
@@ -1488,12 +1561,12 @@
         <f>J7-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="17">
+        <f>K7/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M7" s="16">
         <f>K7-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M7" s="16">
-        <f>L7-($E7*Inputs!$B$7)+($F7*SUM(Inputs!$B$28:$D$28))+($G7*Inputs!$B$12)+($I7*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N7" s="17">
@@ -1501,6 +1574,14 @@
         <v/>
       </c>
       <c r="O7" s="16">
+        <f>M7-(($E7*Inputs!$B$7)+($F7*SUM(Inputs!$B$28:$D$28))+($G7*Inputs!$B$12)+($I7*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P7" s="17">
+        <f>O7/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="16">
         <f>$J$6-J7</f>
         <v/>
       </c>
@@ -1508,14 +1589,14 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Tier 2 — stores 12% / DK-resto 20%</t>
+          <t>Tier 2 — 6m 25% → 6m 20%</t>
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>0.2</v>
+        <v>0.225</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>0.2</v>
+        <v>0.225</v>
       </c>
       <c r="D8" s="20" t="n">
         <v>0.12</v>
@@ -1543,12 +1624,12 @@
         <f>J8-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L8" s="16">
+      <c r="L8" s="17">
+        <f>K8/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M8" s="16">
         <f>K8-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M8" s="16">
-        <f>L8-($E8*Inputs!$B$7)+($F8*SUM(Inputs!$B$28:$D$28))+($G8*Inputs!$B$12)+($I8*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N8" s="17">
@@ -1556,6 +1637,14 @@
         <v/>
       </c>
       <c r="O8" s="16">
+        <f>M8-(($E8*Inputs!$B$7)+($F8*SUM(Inputs!$B$28:$D$28))+($G8*Inputs!$B$12)+($I8*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P8" s="17">
+        <f>O8/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="16">
         <f>$J$6-J8</f>
         <v/>
       </c>
@@ -1563,14 +1652,14 @@
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Tier 3a — stores 12% / DK-resto 16%</t>
+          <t>Tier 3a — 6m 20% → 6m 16%</t>
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="D9" s="20" t="n">
         <v>0.12</v>
@@ -1598,12 +1687,12 @@
         <f>J9-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L9" s="16">
+      <c r="L9" s="17">
+        <f>K9/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M9" s="16">
         <f>K9-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M9" s="16">
-        <f>L9-($E9*Inputs!$B$7)+($F9*SUM(Inputs!$B$28:$D$28))+($G9*Inputs!$B$12)+($I9*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N9" s="17">
@@ -1611,6 +1700,14 @@
         <v/>
       </c>
       <c r="O9" s="16">
+        <f>M9-(($E9*Inputs!$B$7)+($F9*SUM(Inputs!$B$28:$D$28))+($G9*Inputs!$B$12)+($I9*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P9" s="17">
+        <f>O9/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="16">
         <f>$J$6-J9</f>
         <v/>
       </c>
@@ -1618,7 +1715,7 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Tier 3b — shared 16%</t>
+          <t>Tier 3a — 12m stores 12% / DK-resto 16%</t>
         </is>
       </c>
       <c r="B10" s="20" t="n">
@@ -1628,7 +1725,7 @@
         <v>0.16</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>1</v>
@@ -1653,12 +1750,12 @@
         <f>J10-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="17">
+        <f>K10/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M10" s="16">
         <f>K10-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M10" s="16">
-        <f>L10-($E10*Inputs!$B$7)+($F10*SUM(Inputs!$B$28:$D$28))+($G10*Inputs!$B$12)+($I10*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N10" s="17">
@@ -1666,6 +1763,14 @@
         <v/>
       </c>
       <c r="O10" s="16">
+        <f>M10-(($E10*Inputs!$B$7)+($F10*SUM(Inputs!$B$28:$D$28))+($G10*Inputs!$B$12)+($I10*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P10" s="17">
+        <f>O10/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="16">
         <f>$J$6-J10</f>
         <v/>
       </c>
@@ -1673,17 +1778,17 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Revenue-neutral shared 17.50%</t>
+          <t>Tier 3b — 6m tier 2 → 6m shared 16%</t>
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>0.175</v>
+        <v>0.18</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>0.175</v>
+        <v>0.18</v>
       </c>
       <c r="D11" s="20" t="n">
-        <v>0.175</v>
+        <v>0.14</v>
       </c>
       <c r="E11" s="21" t="n">
         <v>1</v>
@@ -1708,12 +1813,12 @@
         <f>J11-SUM(Inputs!$B$24:$D$24)</f>
         <v/>
       </c>
-      <c r="L11" s="16">
+      <c r="L11" s="17">
+        <f>K11/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M11" s="16">
         <f>K11-SUM(Inputs!$B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="M11" s="16">
-        <f>L11-($E11*Inputs!$B$7)+($F11*SUM(Inputs!$B$28:$D$28))+($G11*Inputs!$B$12)+($I11*(Inputs!$B$14+Inputs!$B$15))</f>
         <v/>
       </c>
       <c r="N11" s="17">
@@ -1721,17 +1826,151 @@
         <v/>
       </c>
       <c r="O11" s="16">
+        <f>M11-(($E11*Inputs!$B$7)+($F11*SUM(Inputs!$B$28:$D$28))+($G11*Inputs!$B$12)+($I11*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P11" s="17">
+        <f>O11/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="16">
         <f>$J$6-J11</f>
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Tier 3b — 12m shared 16%</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="16">
+        <f>SUMPRODUCT($B12:$D12,Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="K12" s="16">
+        <f>J12-SUM(Inputs!$B$24:$D$24)</f>
+        <v/>
+      </c>
+      <c r="L12" s="17">
+        <f>K12/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M12" s="16">
+        <f>K12-SUM(Inputs!$B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="N12" s="17">
+        <f>M12/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="O12" s="16">
+        <f>M12-(($E12*Inputs!$B$7)+($F12*SUM(Inputs!$B$28:$D$28))+($G12*Inputs!$B$12)+($I12*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P12" s="17">
+        <f>O12/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="16">
+        <f>$J$6-J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Revenue-neutral shared 17.50%</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="16">
+        <f>SUMPRODUCT($B13:$D13,Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="K13" s="16">
+        <f>J13-SUM(Inputs!$B$24:$D$24)</f>
+        <v/>
+      </c>
+      <c r="L13" s="17">
+        <f>K13/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="M13" s="16">
+        <f>K13-SUM(Inputs!$B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="N13" s="17">
+        <f>M13/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="O13" s="16">
+        <f>M13-(($E13*Inputs!$B$7)+($F13*SUM(Inputs!$B$28:$D$28))+($G13*Inputs!$B$12)+($I13*(Inputs!$B$14+Inputs!$B$15)))</f>
+        <v/>
+      </c>
+      <c r="P13" s="17">
+        <f>O13/SUM(Inputs!$B$21:$D$21)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="16">
+        <f>$J$6-J13</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:O11"/>
+  <autoFilter ref="A5:Q13"/>
   <mergeCells count="2">
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M6:M11">
+  <conditionalFormatting sqref="O6:O13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1750,7 +1989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1776,7 +2015,7 @@
       </c>
       <c r="B3" s="22" t="inlineStr">
         <is>
-          <t>Tier 3b — shared 16%</t>
+          <t>Tier 3b — 12m shared 16%</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1908,15 +2147,15 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>INDEX(Scenarios!$B$6:$B$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))</f>
+        <f>INDEX(Scenarios!$B$6:$B$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))</f>
         <v/>
       </c>
       <c r="C9" s="15">
-        <f>INDEX(Scenarios!$C$6:$C$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))</f>
+        <f>INDEX(Scenarios!$C$6:$C$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>INDEX(Scenarios!$D$6:$D$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))</f>
+        <f>INDEX(Scenarios!$D$6:$D$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))</f>
         <v/>
       </c>
       <c r="E9" s="15">
@@ -2076,15 +2315,15 @@
         </is>
       </c>
       <c r="B15" s="24">
-        <f>IF(=INDEX(Scenarios!$E$6:$E$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,0)</f>
+        <f>IF(=INDEX(Scenarios!$E$6:$E$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,0)</f>
         <v/>
       </c>
       <c r="C15" s="24">
-        <f>IF(=INDEX(Scenarios!$E$6:$E$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,0)</f>
+        <f>IF(=INDEX(Scenarios!$E$6:$E$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,0)</f>
         <v/>
       </c>
       <c r="D15" s="24">
-        <f>IF(=INDEX(Scenarios!$E$6:$E$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$7)</f>
+        <f>IF(=INDEX(Scenarios!$E$6:$E$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$7)</f>
         <v/>
       </c>
       <c r="E15" s="24">
@@ -2104,15 +2343,15 @@
         </is>
       </c>
       <c r="B16" s="24">
-        <f>IF(=INDEX(Scenarios!$F$6:$F$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!B28)</f>
+        <f>IF(=INDEX(Scenarios!$F$6:$F$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!B28)</f>
         <v/>
       </c>
       <c r="C16" s="24">
-        <f>IF(=INDEX(Scenarios!$F$6:$F$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!C28)</f>
+        <f>IF(=INDEX(Scenarios!$F$6:$F$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!C28)</f>
         <v/>
       </c>
       <c r="D16" s="24">
-        <f>IF(=INDEX(Scenarios!$F$6:$F$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!D28)</f>
+        <f>IF(=INDEX(Scenarios!$F$6:$F$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!D28)</f>
         <v/>
       </c>
       <c r="E16" s="24">
@@ -2132,15 +2371,15 @@
         </is>
       </c>
       <c r="B17" s="24">
-        <f>IF(=INDEX(Scenarios!$G$6:$G$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$12*Inputs!B29)</f>
+        <f>IF(=INDEX(Scenarios!$G$6:$G$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$12*Inputs!B29)</f>
         <v/>
       </c>
       <c r="C17" s="24">
-        <f>IF(=INDEX(Scenarios!$G$6:$G$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$12*Inputs!C29)</f>
+        <f>IF(=INDEX(Scenarios!$G$6:$G$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$12*Inputs!C29)</f>
         <v/>
       </c>
       <c r="D17" s="24">
-        <f>IF(=INDEX(Scenarios!$G$6:$G$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$12*Inputs!D29)</f>
+        <f>IF(=INDEX(Scenarios!$G$6:$G$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$12*Inputs!D29)</f>
         <v/>
       </c>
       <c r="E17" s="24">
@@ -2160,15 +2399,15 @@
         </is>
       </c>
       <c r="B18" s="24">
-        <f>IF(=INDEX(Scenarios!$I$6:$I$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!B29)</f>
+        <f>IF(=INDEX(Scenarios!$I$6:$I$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!B29)</f>
         <v/>
       </c>
       <c r="C18" s="24">
-        <f>IF(=INDEX(Scenarios!$I$6:$I$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!C29)</f>
+        <f>IF(=INDEX(Scenarios!$I$6:$I$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!C29)</f>
         <v/>
       </c>
       <c r="D18" s="24">
-        <f>IF(=INDEX(Scenarios!$I$6:$I$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!D29)</f>
+        <f>IF(=INDEX(Scenarios!$I$6:$I$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,(Inputs!$B$14+Inputs!$B$15)*Inputs!D29)</f>
         <v/>
       </c>
       <c r="E18" s="24">
@@ -2244,15 +2483,15 @@
         </is>
       </c>
       <c r="B21" s="16">
-        <f>IF(=INDEX(Scenarios!$H$6:$H$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$13*Inputs!B29)</f>
+        <f>IF(=INDEX(Scenarios!$H$6:$H$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$13*Inputs!B29)</f>
         <v/>
       </c>
       <c r="C21" s="16">
-        <f>IF(=INDEX(Scenarios!$H$6:$H$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$13*Inputs!C29)</f>
+        <f>IF(=INDEX(Scenarios!$H$6:$H$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$13*Inputs!C29)</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>IF(=INDEX(Scenarios!$H$6:$H$11,MATCH($B$3,Scenarios!$A$6:$A$11,0))=0,0,Inputs!$B$13*Inputs!D29)</f>
+        <f>IF(=INDEX(Scenarios!$H$6:$H$13,MATCH($B$3,Scenarios!$A$6:$A$13,0))=0,0,Inputs!$B$13*Inputs!D29)</f>
         <v/>
       </c>
       <c r="E21" s="16">
@@ -2346,6 +2585,34 @@
       <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Baseline commission − selected commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Eater-fee revenue (informational)</t>
+        </is>
+      </c>
+      <c r="B25" s="16">
+        <f>Inputs!B30</f>
+        <v/>
+      </c>
+      <c r="C25" s="16">
+        <f>Inputs!C30</f>
+        <v/>
+      </c>
+      <c r="D25" s="16">
+        <f>Inputs!D30</f>
+        <v/>
+      </c>
+      <c r="E25" s="14">
+        <f>SUM(B25:D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Historical reference only; already included in CP unit economics</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2628,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Scenarios!$A$6:$A$11</formula1>
+      <formula1>=Scenarios!$A$6:$A$13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2370,6 +2637,2260 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:U35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quarterly rate scenarios — editable commission &amp; eater fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Quarter GMV share</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="inlineStr">
+        <is>
+          <t>Edit yellow cells: quarterly GMV shares and commission rates. Eater fees are editable on Inputs row 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DK rate</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Resto rate</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Stores rate</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Eater fees
+info only</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Direct costs</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>CP L1</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>CP L1 %</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>Existing DI</t>
+        </is>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>Historical DF DK/resto
+inside DI</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>CP L2</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>CP L2 %</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>DF campaign
+stores cash</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
+        <is>
+          <t>Bolt+ cash</t>
+        </is>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>PL cash</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>Final cash P&amp;L</t>
+        </is>
+      </c>
+      <c r="U6" s="7" t="inlineStr">
+        <is>
+          <t>Final %</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Tier 1 — 12m 25%</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F7" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G7" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H7" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I7" s="16">
+        <f>C7*Inputs!$B$21*$B$4+D7*Inputs!$C$21*$B$4+E7*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J7" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K7" s="14">
+        <f>I7-J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="25">
+        <f>K7/G7</f>
+        <v/>
+      </c>
+      <c r="M7" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N7" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O7" s="14">
+        <f>K7-M7</f>
+        <v/>
+      </c>
+      <c r="P7" s="25">
+        <f>O7/G7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="24">
+        <f>IF(B7="Q1",Inputs!$B$7/2,IF(B7="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R7" s="24">
+        <f>IF(B7="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B7="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S7" s="24">
+        <f>IF(B7="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T7" s="14">
+        <f>O7-SUM(Q7:S7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="25">
+        <f>T7/G7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 — 12m 25%</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F8" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G8" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H8" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I8" s="16">
+        <f>C8*Inputs!$B$21*$C$4+D8*Inputs!$C$21*$C$4+E8*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J8" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>I8-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="25">
+        <f>K8/G8</f>
+        <v/>
+      </c>
+      <c r="M8" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N8" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O8" s="14">
+        <f>K8-M8</f>
+        <v/>
+      </c>
+      <c r="P8" s="25">
+        <f>O8/G8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="24">
+        <f>IF(B8="Q1",Inputs!$B$7/2,IF(B8="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R8" s="24">
+        <f>IF(B8="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B8="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S8" s="24">
+        <f>IF(B8="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T8" s="14">
+        <f>O8-SUM(Q8:S8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="25">
+        <f>T8/G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 — 12m 25%</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F9" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G9" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H9" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I9" s="16">
+        <f>C9*Inputs!$B$21*$D$4+D9*Inputs!$C$21*$D$4+E9*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K9" s="14">
+        <f>I9-J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="25">
+        <f>K9/G9</f>
+        <v/>
+      </c>
+      <c r="M9" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N9" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O9" s="14">
+        <f>K9-M9</f>
+        <v/>
+      </c>
+      <c r="P9" s="25">
+        <f>O9/G9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="24">
+        <f>IF(B9="Q1",Inputs!$B$7/2,IF(B9="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R9" s="24">
+        <f>IF(B9="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B9="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S9" s="24">
+        <f>IF(B9="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T9" s="14">
+        <f>O9-SUM(Q9:S9)</f>
+        <v/>
+      </c>
+      <c r="U9" s="25">
+        <f>T9/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 — 12m 25%</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F10" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G10" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H10" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I10" s="16">
+        <f>C10*Inputs!$B$21*$E$4+D10*Inputs!$C$21*$E$4+E10*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K10" s="14">
+        <f>I10-J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="25">
+        <f>K10/G10</f>
+        <v/>
+      </c>
+      <c r="M10" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N10" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O10" s="14">
+        <f>K10-M10</f>
+        <v/>
+      </c>
+      <c r="P10" s="25">
+        <f>O10/G10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="24">
+        <f>IF(B10="Q1",Inputs!$B$7/2,IF(B10="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R10" s="24">
+        <f>IF(B10="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B10="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S10" s="24">
+        <f>IF(B10="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T10" s="14">
+        <f>O10-SUM(Q10:S10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="25">
+        <f>T10/G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Tier 2 — 6m 25% → 6m 20%</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F12" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G12" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H12" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I12" s="16">
+        <f>C12*Inputs!$B$21*$B$4+D12*Inputs!$C$21*$B$4+E12*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J12" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K12" s="14">
+        <f>I12-J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="25">
+        <f>K12/G12</f>
+        <v/>
+      </c>
+      <c r="M12" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N12" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O12" s="14">
+        <f>K12-M12</f>
+        <v/>
+      </c>
+      <c r="P12" s="25">
+        <f>O12/G12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="24">
+        <f>IF(B12="Q1",Inputs!$B$7/2,IF(B12="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R12" s="24">
+        <f>IF(B12="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B12="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S12" s="24">
+        <f>IF(B12="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T12" s="14">
+        <f>O12-SUM(Q12:S12)</f>
+        <v/>
+      </c>
+      <c r="U12" s="25">
+        <f>T12/G12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Tier 2 — 6m 25% → 6m 20%</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F13" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G13" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H13" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I13" s="16">
+        <f>C13*Inputs!$B$21*$C$4+D13*Inputs!$C$21*$C$4+E13*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J13" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K13" s="14">
+        <f>I13-J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="25">
+        <f>K13/G13</f>
+        <v/>
+      </c>
+      <c r="M13" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N13" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O13" s="14">
+        <f>K13-M13</f>
+        <v/>
+      </c>
+      <c r="P13" s="25">
+        <f>O13/G13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="24">
+        <f>IF(B13="Q1",Inputs!$B$7/2,IF(B13="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R13" s="24">
+        <f>IF(B13="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B13="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S13" s="24">
+        <f>IF(B13="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T13" s="14">
+        <f>O13-SUM(Q13:S13)</f>
+        <v/>
+      </c>
+      <c r="U13" s="25">
+        <f>T13/G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Tier 2 — 6m 25% → 6m 20%</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F14" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G14" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H14" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I14" s="16">
+        <f>C14*Inputs!$B$21*$D$4+D14*Inputs!$C$21*$D$4+E14*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J14" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K14" s="14">
+        <f>I14-J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="25">
+        <f>K14/G14</f>
+        <v/>
+      </c>
+      <c r="M14" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N14" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O14" s="14">
+        <f>K14-M14</f>
+        <v/>
+      </c>
+      <c r="P14" s="25">
+        <f>O14/G14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="24">
+        <f>IF(B14="Q1",Inputs!$B$7/2,IF(B14="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R14" s="24">
+        <f>IF(B14="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B14="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S14" s="24">
+        <f>IF(B14="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T14" s="14">
+        <f>O14-SUM(Q14:S14)</f>
+        <v/>
+      </c>
+      <c r="U14" s="25">
+        <f>T14/G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Tier 2 — 6m 25% → 6m 20%</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F15" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G15" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H15" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I15" s="16">
+        <f>C15*Inputs!$B$21*$E$4+D15*Inputs!$C$21*$E$4+E15*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J15" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K15" s="14">
+        <f>I15-J15</f>
+        <v/>
+      </c>
+      <c r="L15" s="25">
+        <f>K15/G15</f>
+        <v/>
+      </c>
+      <c r="M15" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N15" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O15" s="14">
+        <f>K15-M15</f>
+        <v/>
+      </c>
+      <c r="P15" s="25">
+        <f>O15/G15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="24">
+        <f>IF(B15="Q1",Inputs!$B$7/2,IF(B15="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R15" s="24">
+        <f>IF(B15="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B15="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S15" s="24">
+        <f>IF(B15="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T15" s="14">
+        <f>O15-SUM(Q15:S15)</f>
+        <v/>
+      </c>
+      <c r="U15" s="25">
+        <f>T15/G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Tier 3a — 6m 20% → 6m 16%</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F17" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G17" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H17" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I17" s="16">
+        <f>C17*Inputs!$B$21*$B$4+D17*Inputs!$C$21*$B$4+E17*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K17" s="14">
+        <f>I17-J17</f>
+        <v/>
+      </c>
+      <c r="L17" s="25">
+        <f>K17/G17</f>
+        <v/>
+      </c>
+      <c r="M17" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N17" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O17" s="14">
+        <f>K17-M17</f>
+        <v/>
+      </c>
+      <c r="P17" s="25">
+        <f>O17/G17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="24">
+        <f>IF(B17="Q1",Inputs!$B$7/2,IF(B17="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R17" s="24">
+        <f>IF(B17="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B17="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S17" s="24">
+        <f>IF(B17="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T17" s="14">
+        <f>O17-SUM(Q17:S17)</f>
+        <v/>
+      </c>
+      <c r="U17" s="25">
+        <f>T17/G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 6m 20% → 6m 16%</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F18" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G18" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H18" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I18" s="16">
+        <f>C18*Inputs!$B$21*$C$4+D18*Inputs!$C$21*$C$4+E18*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J18" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K18" s="14">
+        <f>I18-J18</f>
+        <v/>
+      </c>
+      <c r="L18" s="25">
+        <f>K18/G18</f>
+        <v/>
+      </c>
+      <c r="M18" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N18" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O18" s="14">
+        <f>K18-M18</f>
+        <v/>
+      </c>
+      <c r="P18" s="25">
+        <f>O18/G18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="24">
+        <f>IF(B18="Q1",Inputs!$B$7/2,IF(B18="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R18" s="24">
+        <f>IF(B18="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B18="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S18" s="24">
+        <f>IF(B18="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T18" s="14">
+        <f>O18-SUM(Q18:S18)</f>
+        <v/>
+      </c>
+      <c r="U18" s="25">
+        <f>T18/G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 6m 20% → 6m 16%</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F19" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H19" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I19" s="16">
+        <f>C19*Inputs!$B$21*$D$4+D19*Inputs!$C$21*$D$4+E19*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K19" s="14">
+        <f>I19-J19</f>
+        <v/>
+      </c>
+      <c r="L19" s="25">
+        <f>K19/G19</f>
+        <v/>
+      </c>
+      <c r="M19" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N19" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O19" s="14">
+        <f>K19-M19</f>
+        <v/>
+      </c>
+      <c r="P19" s="25">
+        <f>O19/G19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="24">
+        <f>IF(B19="Q1",Inputs!$B$7/2,IF(B19="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R19" s="24">
+        <f>IF(B19="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B19="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S19" s="24">
+        <f>IF(B19="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T19" s="14">
+        <f>O19-SUM(Q19:S19)</f>
+        <v/>
+      </c>
+      <c r="U19" s="25">
+        <f>T19/G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 6m 20% → 6m 16%</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F20" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G20" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H20" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I20" s="16">
+        <f>C20*Inputs!$B$21*$E$4+D20*Inputs!$C$21*$E$4+E20*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J20" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K20" s="14">
+        <f>I20-J20</f>
+        <v/>
+      </c>
+      <c r="L20" s="25">
+        <f>K20/G20</f>
+        <v/>
+      </c>
+      <c r="M20" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N20" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O20" s="14">
+        <f>K20-M20</f>
+        <v/>
+      </c>
+      <c r="P20" s="25">
+        <f>O20/G20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="24">
+        <f>IF(B20="Q1",Inputs!$B$7/2,IF(B20="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R20" s="24">
+        <f>IF(B20="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B20="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S20" s="24">
+        <f>IF(B20="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T20" s="14">
+        <f>O20-SUM(Q20:S20)</f>
+        <v/>
+      </c>
+      <c r="U20" s="25">
+        <f>T20/G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Tier 3a — 12m DK/resto 16%</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F22" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H22" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I22" s="16">
+        <f>C22*Inputs!$B$21*$B$4+D22*Inputs!$C$21*$B$4+E22*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J22" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K22" s="14">
+        <f>I22-J22</f>
+        <v/>
+      </c>
+      <c r="L22" s="25">
+        <f>K22/G22</f>
+        <v/>
+      </c>
+      <c r="M22" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N22" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O22" s="14">
+        <f>K22-M22</f>
+        <v/>
+      </c>
+      <c r="P22" s="25">
+        <f>O22/G22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="24">
+        <f>IF(B22="Q1",Inputs!$B$7/2,IF(B22="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R22" s="24">
+        <f>IF(B22="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B22="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S22" s="24">
+        <f>IF(B22="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T22" s="14">
+        <f>O22-SUM(Q22:S22)</f>
+        <v/>
+      </c>
+      <c r="U22" s="25">
+        <f>T22/G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 12m DK/resto 16%</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F23" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G23" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H23" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I23" s="16">
+        <f>C23*Inputs!$B$21*$C$4+D23*Inputs!$C$21*$C$4+E23*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J23" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K23" s="14">
+        <f>I23-J23</f>
+        <v/>
+      </c>
+      <c r="L23" s="25">
+        <f>K23/G23</f>
+        <v/>
+      </c>
+      <c r="M23" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N23" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O23" s="14">
+        <f>K23-M23</f>
+        <v/>
+      </c>
+      <c r="P23" s="25">
+        <f>O23/G23</f>
+        <v/>
+      </c>
+      <c r="Q23" s="24">
+        <f>IF(B23="Q1",Inputs!$B$7/2,IF(B23="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R23" s="24">
+        <f>IF(B23="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B23="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S23" s="24">
+        <f>IF(B23="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T23" s="14">
+        <f>O23-SUM(Q23:S23)</f>
+        <v/>
+      </c>
+      <c r="U23" s="25">
+        <f>T23/G23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 12m DK/resto 16%</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F24" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G24" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H24" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I24" s="16">
+        <f>C24*Inputs!$B$21*$D$4+D24*Inputs!$C$21*$D$4+E24*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J24" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K24" s="14">
+        <f>I24-J24</f>
+        <v/>
+      </c>
+      <c r="L24" s="25">
+        <f>K24/G24</f>
+        <v/>
+      </c>
+      <c r="M24" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N24" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O24" s="14">
+        <f>K24-M24</f>
+        <v/>
+      </c>
+      <c r="P24" s="25">
+        <f>O24/G24</f>
+        <v/>
+      </c>
+      <c r="Q24" s="24">
+        <f>IF(B24="Q1",Inputs!$B$7/2,IF(B24="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R24" s="24">
+        <f>IF(B24="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B24="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S24" s="24">
+        <f>IF(B24="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T24" s="14">
+        <f>O24-SUM(Q24:S24)</f>
+        <v/>
+      </c>
+      <c r="U24" s="25">
+        <f>T24/G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3a — 12m DK/resto 16%</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F25" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H25" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I25" s="16">
+        <f>C25*Inputs!$B$21*$E$4+D25*Inputs!$C$21*$E$4+E25*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J25" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K25" s="14">
+        <f>I25-J25</f>
+        <v/>
+      </c>
+      <c r="L25" s="25">
+        <f>K25/G25</f>
+        <v/>
+      </c>
+      <c r="M25" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N25" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O25" s="14">
+        <f>K25-M25</f>
+        <v/>
+      </c>
+      <c r="P25" s="25">
+        <f>O25/G25</f>
+        <v/>
+      </c>
+      <c r="Q25" s="24">
+        <f>IF(B25="Q1",Inputs!$B$7/2,IF(B25="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R25" s="24">
+        <f>IF(B25="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B25="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S25" s="24">
+        <f>IF(B25="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T25" s="14">
+        <f>O25-SUM(Q25:S25)</f>
+        <v/>
+      </c>
+      <c r="U25" s="25">
+        <f>T25/G25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Tier 3b — 6m tier 2 → 6m shared 16%</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F27" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G27" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H27" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I27" s="16">
+        <f>C27*Inputs!$B$21*$B$4+D27*Inputs!$C$21*$B$4+E27*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J27" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K27" s="14">
+        <f>I27-J27</f>
+        <v/>
+      </c>
+      <c r="L27" s="25">
+        <f>K27/G27</f>
+        <v/>
+      </c>
+      <c r="M27" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N27" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O27" s="14">
+        <f>K27-M27</f>
+        <v/>
+      </c>
+      <c r="P27" s="25">
+        <f>O27/G27</f>
+        <v/>
+      </c>
+      <c r="Q27" s="24">
+        <f>IF(B27="Q1",Inputs!$B$7/2,IF(B27="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R27" s="24">
+        <f>IF(B27="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B27="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S27" s="24">
+        <f>IF(B27="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T27" s="14">
+        <f>O27-SUM(Q27:S27)</f>
+        <v/>
+      </c>
+      <c r="U27" s="25">
+        <f>T27/G27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 6m tier 2 → 6m shared 16%</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F28" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G28" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H28" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I28" s="16">
+        <f>C28*Inputs!$B$21*$C$4+D28*Inputs!$C$21*$C$4+E28*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J28" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K28" s="14">
+        <f>I28-J28</f>
+        <v/>
+      </c>
+      <c r="L28" s="25">
+        <f>K28/G28</f>
+        <v/>
+      </c>
+      <c r="M28" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N28" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O28" s="14">
+        <f>K28-M28</f>
+        <v/>
+      </c>
+      <c r="P28" s="25">
+        <f>O28/G28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="24">
+        <f>IF(B28="Q1",Inputs!$B$7/2,IF(B28="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R28" s="24">
+        <f>IF(B28="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B28="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S28" s="24">
+        <f>IF(B28="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T28" s="14">
+        <f>O28-SUM(Q28:S28)</f>
+        <v/>
+      </c>
+      <c r="U28" s="25">
+        <f>T28/G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 6m tier 2 → 6m shared 16%</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F29" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H29" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I29" s="16">
+        <f>C29*Inputs!$B$21*$D$4+D29*Inputs!$C$21*$D$4+E29*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J29" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K29" s="14">
+        <f>I29-J29</f>
+        <v/>
+      </c>
+      <c r="L29" s="25">
+        <f>K29/G29</f>
+        <v/>
+      </c>
+      <c r="M29" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N29" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O29" s="14">
+        <f>K29-M29</f>
+        <v/>
+      </c>
+      <c r="P29" s="25">
+        <f>O29/G29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="24">
+        <f>IF(B29="Q1",Inputs!$B$7/2,IF(B29="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R29" s="24">
+        <f>IF(B29="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B29="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S29" s="24">
+        <f>IF(B29="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T29" s="14">
+        <f>O29-SUM(Q29:S29)</f>
+        <v/>
+      </c>
+      <c r="U29" s="25">
+        <f>T29/G29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 6m tier 2 → 6m shared 16%</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F30" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G30" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H30" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I30" s="16">
+        <f>C30*Inputs!$B$21*$E$4+D30*Inputs!$C$21*$E$4+E30*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J30" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K30" s="14">
+        <f>I30-J30</f>
+        <v/>
+      </c>
+      <c r="L30" s="25">
+        <f>K30/G30</f>
+        <v/>
+      </c>
+      <c r="M30" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N30" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O30" s="14">
+        <f>K30-M30</f>
+        <v/>
+      </c>
+      <c r="P30" s="25">
+        <f>O30/G30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="24">
+        <f>IF(B30="Q1",Inputs!$B$7/2,IF(B30="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R30" s="24">
+        <f>IF(B30="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B30="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S30" s="24">
+        <f>IF(B30="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T30" s="14">
+        <f>O30-SUM(Q30:S30)</f>
+        <v/>
+      </c>
+      <c r="U30" s="25">
+        <f>T30/G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>Tier 3b — 12m shared 16%</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F32" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$B$4</f>
+        <v/>
+      </c>
+      <c r="G32" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$B$4</f>
+        <v/>
+      </c>
+      <c r="H32" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$B$4</f>
+        <v/>
+      </c>
+      <c r="I32" s="16">
+        <f>C32*Inputs!$B$21*$B$4+D32*Inputs!$C$21*$B$4+E32*Inputs!$D$21*$B$4</f>
+        <v/>
+      </c>
+      <c r="J32" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$B$4</f>
+        <v/>
+      </c>
+      <c r="K32" s="14">
+        <f>I32-J32</f>
+        <v/>
+      </c>
+      <c r="L32" s="25">
+        <f>K32/G32</f>
+        <v/>
+      </c>
+      <c r="M32" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$B$4</f>
+        <v/>
+      </c>
+      <c r="N32" s="24">
+        <f>Inputs!$B$16*$B$4</f>
+        <v/>
+      </c>
+      <c r="O32" s="14">
+        <f>K32-M32</f>
+        <v/>
+      </c>
+      <c r="P32" s="25">
+        <f>O32/G32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="24">
+        <f>IF(B32="Q1",Inputs!$B$7/2,IF(B32="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R32" s="24">
+        <f>IF(B32="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B32="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S32" s="24">
+        <f>IF(B32="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T32" s="14">
+        <f>O32-SUM(Q32:S32)</f>
+        <v/>
+      </c>
+      <c r="U32" s="25">
+        <f>T32/G32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 12m shared 16%</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F33" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$C$4</f>
+        <v/>
+      </c>
+      <c r="G33" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$C$4</f>
+        <v/>
+      </c>
+      <c r="H33" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$C$4</f>
+        <v/>
+      </c>
+      <c r="I33" s="16">
+        <f>C33*Inputs!$B$21*$C$4+D33*Inputs!$C$21*$C$4+E33*Inputs!$D$21*$C$4</f>
+        <v/>
+      </c>
+      <c r="J33" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$C$4</f>
+        <v/>
+      </c>
+      <c r="K33" s="14">
+        <f>I33-J33</f>
+        <v/>
+      </c>
+      <c r="L33" s="25">
+        <f>K33/G33</f>
+        <v/>
+      </c>
+      <c r="M33" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$C$4</f>
+        <v/>
+      </c>
+      <c r="N33" s="24">
+        <f>Inputs!$B$16*$C$4</f>
+        <v/>
+      </c>
+      <c r="O33" s="14">
+        <f>K33-M33</f>
+        <v/>
+      </c>
+      <c r="P33" s="25">
+        <f>O33/G33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="24">
+        <f>IF(B33="Q1",Inputs!$B$7/2,IF(B33="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R33" s="24">
+        <f>IF(B33="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B33="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S33" s="24">
+        <f>IF(B33="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T33" s="14">
+        <f>O33-SUM(Q33:S33)</f>
+        <v/>
+      </c>
+      <c r="U33" s="25">
+        <f>T33/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 12m shared 16%</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F34" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$D$4</f>
+        <v/>
+      </c>
+      <c r="G34" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$D$4</f>
+        <v/>
+      </c>
+      <c r="H34" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$D$4</f>
+        <v/>
+      </c>
+      <c r="I34" s="16">
+        <f>C34*Inputs!$B$21*$D$4+D34*Inputs!$C$21*$D$4+E34*Inputs!$D$21*$D$4</f>
+        <v/>
+      </c>
+      <c r="J34" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$D$4</f>
+        <v/>
+      </c>
+      <c r="K34" s="14">
+        <f>I34-J34</f>
+        <v/>
+      </c>
+      <c r="L34" s="25">
+        <f>K34/G34</f>
+        <v/>
+      </c>
+      <c r="M34" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$D$4</f>
+        <v/>
+      </c>
+      <c r="N34" s="24">
+        <f>Inputs!$B$16*$D$4</f>
+        <v/>
+      </c>
+      <c r="O34" s="14">
+        <f>K34-M34</f>
+        <v/>
+      </c>
+      <c r="P34" s="25">
+        <f>O34/G34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="24">
+        <f>IF(B34="Q1",Inputs!$B$7/2,IF(B34="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R34" s="24">
+        <f>IF(B34="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B34="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S34" s="24">
+        <f>IF(B34="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T34" s="14">
+        <f>O34-SUM(Q34:S34)</f>
+        <v/>
+      </c>
+      <c r="U34" s="25">
+        <f>T34/G34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Tier 3b — 12m shared 16%</t>
+        </is>
+      </c>
+      <c r="B35" s="28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F35" s="12">
+        <f>SUM(Inputs!$B$20:$D$20)*$E$4</f>
+        <v/>
+      </c>
+      <c r="G35" s="16">
+        <f>SUM(Inputs!$B$21:$D$21)*$E$4</f>
+        <v/>
+      </c>
+      <c r="H35" s="16">
+        <f>SUM(Inputs!$B$30:$D$30)*$E$4</f>
+        <v/>
+      </c>
+      <c r="I35" s="16">
+        <f>C35*Inputs!$B$21*$E$4+D35*Inputs!$C$21*$E$4+E35*Inputs!$D$21*$E$4</f>
+        <v/>
+      </c>
+      <c r="J35" s="16">
+        <f>SUM(Inputs!$B$24:$D$24)*$E$4</f>
+        <v/>
+      </c>
+      <c r="K35" s="14">
+        <f>I35-J35</f>
+        <v/>
+      </c>
+      <c r="L35" s="25">
+        <f>K35/G35</f>
+        <v/>
+      </c>
+      <c r="M35" s="16">
+        <f>SUM(Inputs!$B$26:$D$26)*$E$4</f>
+        <v/>
+      </c>
+      <c r="N35" s="24">
+        <f>Inputs!$B$16*$E$4</f>
+        <v/>
+      </c>
+      <c r="O35" s="14">
+        <f>K35-M35</f>
+        <v/>
+      </c>
+      <c r="P35" s="25">
+        <f>O35/G35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="24">
+        <f>IF(B35="Q1",Inputs!$B$7/2,IF(B35="Q2",Inputs!$B$7/2,0))</f>
+        <v/>
+      </c>
+      <c r="R35" s="24">
+        <f>IF(B35="Q1",SUM(Inputs!$B$28:$D$28)/2,IF(B35="Q2",SUM(Inputs!$B$28:$D$28)/2,0))</f>
+        <v/>
+      </c>
+      <c r="S35" s="24">
+        <f>IF(B35="Q1",Inputs!$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="T35" s="14">
+        <f>O35-SUM(Q35:S35)</f>
+        <v/>
+      </c>
+      <c r="U35" s="25">
+        <f>T35/G35</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:U35"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="F3:U4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="T7:T35">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2758,7 +5279,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2847,22 +5368,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>silpo-culinary-scenarios</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Offer thresholds and scenarios</t>
         </is>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
         <is>
           <t>GitHub Pages v6a97416</t>
         </is>
       </c>
-      <c r="D7" s="27" t="inlineStr">
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>Rates/thresholds reflected in Scenarios</t>
         </is>

</xml_diff>

<commit_message>
Model tier volumes and cost comments in calculator
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Silpo_2027_DK_Resto_Stores_PnL_Calculator.xlsx
+++ b/Silpo_2027_DK_Resto_Stores_PnL_Calculator.xlsx
@@ -15,14 +15,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'P&amp;L by vertical'!$A$5:$U$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Scenarios!$A$5:$AA$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Scenarios!$A$5:$AF$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="140">
   <si>
     <t>Silpo 2027 — DK, Resto &amp; Stores P&amp;L calculator</t>
   </si>
@@ -268,46 +268,64 @@
     <t>Partner saving</t>
   </si>
   <si>
+    <t>Eater fee € / order</t>
+  </si>
+  <si>
+    <t>Eater fee % GMV</t>
+  </si>
+  <si>
+    <t>Direct costs include</t>
+  </si>
+  <si>
+    <t>Stores orders</t>
+  </si>
+  <si>
+    <t>Stores GMV</t>
+  </si>
+  <si>
     <t>Current effective rates</t>
   </si>
   <si>
     <t>Current historical / Shared16 stores</t>
   </si>
   <si>
+    <t>CPO / courier; demand, supply &amp; fraud refunds; payment processing; bad debt; operations &amp; customer support. Excludes DI and incremental promo.</t>
+  </si>
+  <si>
     <t>Tier 1 · launch</t>
   </si>
   <si>
-    <t>12 months at launch rates</t>
+    <t>12m launch. Фіксувати комісію на 2 роки.</t>
   </si>
   <si>
     <t>Tier 2 · €33k stores GMV / month</t>
   </si>
   <si>
-    <t>6m DK/resto 25%, then 6m 20%; threshold €33k</t>
+    <t>6m DK/resto 25%, 6m 20%; поріг €33k. E-zoo activation: commission ≥15% + Біла ромашка.</t>
   </si>
   <si>
     <t>Tier 3a · step-down to 16%</t>
   </si>
   <si>
-    <t>6m DK/resto 20%, then 6m 16%; stores stays 12%</t>
+    <t>6m DK/resto 20%, then 6m 16%; stores 12%. Resto буде неприбутковим і не зможе інвестувати в smart promo.</t>
   </si>
   <si>
     <t>Tier 3a · 12m DK/resto 16%</t>
   </si>
   <si>
-    <t>12 months: stores 12%, DK/resto 16%</t>
+    <t>12m stores 12% / DK-resto 16%. Resto буде неприбутковим і не зможе інвестувати в smart promo.</t>
   </si>
   <si>
     <t>Tier 3b · step to shared 16%</t>
   </si>
   <si>
-    <t>6m tier 2, then 6m shared 16%</t>
+    <t>6m Tier 2, then 6m shared 16%. Resto буде неприбутковим і не зможе інвестувати в smart promo.</t>
   </si>
   <si>
     <t>Tier 3b · 12m shared 16%</t>
   </si>
   <si>
-    <t>12 months shared 16%</t>
+    <t>12m shared 16%. Resto буде неприбутковим і не зможе інвестувати в smart promo.</t>
   </si>
   <si>
     <t>P&amp;L by vertical — all annual scenarios</t>
@@ -1512,17 +1530,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AF12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
     <col min="2" max="7" width="11.7109375" customWidth="1"/>
     <col min="8" max="8" width="15.7109375" customWidth="1"/>
     <col min="9" max="9" width="38.7109375" customWidth="1"/>
-    <col min="10" max="27" width="15.7109375" customWidth="1"/>
+    <col min="10" max="29" width="15.7109375" customWidth="1"/>
+    <col min="30" max="30" width="52.7109375" customWidth="1"/>
+    <col min="31" max="32" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:32">
       <c r="A1" s="1" t="s">
         <v>52</v>
       </c>
@@ -1552,7 +1572,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:32">
       <c r="A3" s="4" t="s">
         <v>53</v>
       </c>
@@ -1582,7 +1602,7 @@
       <c r="Y3" s="4"/>
       <c r="Z3" s="4"/>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:32">
       <c r="A5" s="5" t="s">
         <v>54</v>
       </c>
@@ -1664,10 +1684,25 @@
       <c r="AA5" s="5" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="6" spans="1:27">
+      <c r="AB5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD5" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AE5" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF5" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B6" s="12">
         <v>0.2013996822249659</v>
@@ -1691,26 +1726,26 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J6" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
+        <f>SUM(Inputs!$B$28:$C$28)+AE6</f>
         <v>109290</v>
       </c>
       <c r="K6" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
+        <f>SUM(Inputs!$B$29:$C$29)+AF6</f>
         <v>1915828.04</v>
       </c>
       <c r="L6" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE6/Inputs!$D$28</f>
         <v>216051.47</v>
       </c>
       <c r="M6" s="11">
-        <f>Inputs!$B$29*(B6+C6)/2+Inputs!$C$29*(D6+E6)/2+Inputs!$D$29*(F6+G6)/2</f>
+        <f>Inputs!$B$29*(B6+C6)/2+Inputs!$C$29*(D6+E6)/2+AF6*(F6+G6)/2</f>
         <v>351356.37</v>
       </c>
       <c r="N6" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE6/Inputs!$D$28</f>
         <v>363478.82355999993</v>
       </c>
       <c r="O6" s="10">
@@ -1722,7 +1757,7 @@
         <v>0.10644432181919627</v>
       </c>
       <c r="Q6" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE6/Inputs!$D$28</f>
         <v>129749.6</v>
       </c>
       <c r="R6" s="15">
@@ -1738,11 +1773,11 @@
         <v>0.03871924561663688</v>
       </c>
       <c r="U6" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(AE6=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="V6" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
+        <f>Inputs!$B$9+IF(AE6=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>25415.45</v>
       </c>
       <c r="W6" s="15">
@@ -1765,10 +1800,27 @@
         <f>$M$6-M6</f>
         <v>-15482.880000000005</v>
       </c>
-    </row>
-    <row r="7" spans="1:27">
+      <c r="AB6" s="11">
+        <f>L6/J6</f>
+        <v>1.9768640314758898</v>
+      </c>
+      <c r="AC6" s="13">
+        <f>L6/K6</f>
+        <v>0.1127718487719806</v>
+      </c>
+      <c r="AD6" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE6" s="8">
+        <v>50400</v>
+      </c>
+      <c r="AF6" s="7">
+        <v>852768</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32">
       <c r="A7" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B7" s="12">
         <v>0.25</v>
@@ -1792,39 +1844,39 @@
         <v>0</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="J7" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
-        <v>109290</v>
+        <f>SUM(Inputs!$B$28:$C$28)+AE7</f>
+        <v>89500</v>
       </c>
       <c r="K7" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
-        <v>1915828.04</v>
+        <f>SUM(Inputs!$B$29:$C$29)+AF7</f>
+        <v>1490860.04</v>
       </c>
       <c r="L7" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
-        <v>216051.47</v>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE7/Inputs!$D$28</f>
+        <v>178054.66999999998</v>
       </c>
       <c r="M7" s="11">
-        <f>Inputs!$B$29*(B7+C7)/2+Inputs!$C$29*(D7+E7)/2+Inputs!$D$29*(F7+G7)/2</f>
-        <v>368097.17</v>
+        <f>Inputs!$B$29*(B7+C7)/2+Inputs!$C$29*(D7+E7)/2+AF7*(F7+G7)/2</f>
+        <v>317101.01</v>
       </c>
       <c r="N7" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
-        <v>363478.82355999993</v>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE7/Inputs!$D$28</f>
+        <v>296178.0150014206</v>
       </c>
       <c r="O7" s="10">
         <f>M7-N7+L7</f>
-        <v>220669.81644000008</v>
+        <v>198977.66499857942</v>
       </c>
       <c r="P7" s="14">
         <f>O7/K7</f>
-        <v>0.11518247558376903</v>
+        <v>0.13346501996161855</v>
       </c>
       <c r="Q7" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
-        <v>129749.6</v>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE7/Inputs!$D$28</f>
+        <v>118469.3</v>
       </c>
       <c r="R7" s="15">
         <f>Inputs!$B$8</f>
@@ -1832,19 +1884,19 @@
       </c>
       <c r="S7" s="10">
         <f>O7-Q7</f>
-        <v>90920.21644000008</v>
+        <v>80508.36499857942</v>
       </c>
       <c r="T7" s="14">
         <f>S7/K7</f>
-        <v>0.04745739938120964</v>
+        <v>0.05400128975123608</v>
       </c>
       <c r="U7" s="15">
-        <f>Inputs!$B$7</f>
-        <v>28000</v>
+        <f>IF(AE7=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
+        <v>14000</v>
       </c>
       <c r="V7" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
-        <v>25415.45</v>
+        <f>Inputs!$B$9+IF(AE7=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
+        <v>20015.45</v>
       </c>
       <c r="W7" s="15">
         <f>Inputs!$B$11</f>
@@ -1852,11 +1904,11 @@
       </c>
       <c r="X7" s="10">
         <f>S7-SUM(U7:W7)</f>
-        <v>27504.76644000008</v>
+        <v>36492.91499857942</v>
       </c>
       <c r="Y7" s="14">
         <f>X7/K7</f>
-        <v>0.014356594572026453</v>
+        <v>0.02447776050029446</v>
       </c>
       <c r="Z7" s="11">
         <f>Inputs!$B$12</f>
@@ -1864,12 +1916,29 @@
       </c>
       <c r="AA7" s="11">
         <f>$M$6-M7</f>
-        <v>-32223.679999999993</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27">
+        <v>18772.47999999998</v>
+      </c>
+      <c r="AB7" s="11">
+        <f>L7/J7</f>
+        <v>1.9894376536312848</v>
+      </c>
+      <c r="AC7" s="13">
+        <f>L7/K7</f>
+        <v>0.11943084207958245</v>
+      </c>
+      <c r="AD7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE7" s="8">
+        <v>30610</v>
+      </c>
+      <c r="AF7" s="7">
+        <v>427800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
       <c r="A8" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B8" s="12">
         <v>0.25</v>
@@ -1893,39 +1962,39 @@
         <v>33000</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="J8" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
-        <v>109290</v>
+        <f>SUM(Inputs!$B$28:$C$28)+AE8</f>
+        <v>89500</v>
       </c>
       <c r="K8" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
-        <v>1915828.04</v>
+        <f>SUM(Inputs!$B$29:$C$29)+AF8</f>
+        <v>1490860.04</v>
       </c>
       <c r="L8" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
-        <v>216051.47</v>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE8/Inputs!$D$28</f>
+        <v>178054.66999999998</v>
       </c>
       <c r="M8" s="11">
-        <f>Inputs!$B$29*(B8+C8)/2+Inputs!$C$29*(D8+E8)/2+Inputs!$D$29*(F8+G8)/2</f>
-        <v>341520.669</v>
+        <f>Inputs!$B$29*(B8+C8)/2+Inputs!$C$29*(D8+E8)/2+AF8*(F8+G8)/2</f>
+        <v>290524.50899999996</v>
       </c>
       <c r="N8" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
-        <v>363478.82355999993</v>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE8/Inputs!$D$28</f>
+        <v>296178.0150014206</v>
       </c>
       <c r="O8" s="10">
         <f>M8-N8+L8</f>
-        <v>194093.31544000003</v>
+        <v>172401.16399857937</v>
       </c>
       <c r="P8" s="14">
         <f>O8/K8</f>
-        <v>0.10131040541613538</v>
+        <v>0.11563873158648706</v>
       </c>
       <c r="Q8" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
-        <v>129749.6</v>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE8/Inputs!$D$28</f>
+        <v>118469.3</v>
       </c>
       <c r="R8" s="15">
         <f>Inputs!$B$8</f>
@@ -1933,19 +2002,19 @@
       </c>
       <c r="S8" s="10">
         <f>O8-Q8</f>
-        <v>64343.71544000003</v>
+        <v>53931.86399857937</v>
       </c>
       <c r="T8" s="14">
         <f>S8/K8</f>
-        <v>0.03358532921357599</v>
+        <v>0.036175001376104604</v>
       </c>
       <c r="U8" s="15">
-        <f>Inputs!$B$7</f>
-        <v>28000</v>
+        <f>IF(AE8=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
+        <v>14000</v>
       </c>
       <c r="V8" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
-        <v>25415.45</v>
+        <f>Inputs!$B$9+IF(AE8=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
+        <v>20015.45</v>
       </c>
       <c r="W8" s="15">
         <f>Inputs!$B$11</f>
@@ -1953,11 +2022,11 @@
       </c>
       <c r="X8" s="10">
         <f>S8-SUM(U8:W8)</f>
-        <v>928.2654400000283</v>
+        <v>9916.41399857937</v>
       </c>
       <c r="Y8" s="14">
         <f>X8/K8</f>
-        <v>0.0004845244043928015</v>
+        <v>0.006651472125162983</v>
       </c>
       <c r="Z8" s="11">
         <f>Inputs!$B$12</f>
@@ -1965,12 +2034,29 @@
       </c>
       <c r="AA8" s="11">
         <f>$M$6-M8</f>
-        <v>-5647.179000000004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27">
+        <v>45348.98100000003</v>
+      </c>
+      <c r="AB8" s="11">
+        <f>L8/J8</f>
+        <v>1.9894376536312848</v>
+      </c>
+      <c r="AC8" s="13">
+        <f>L8/K8</f>
+        <v>0.11943084207958245</v>
+      </c>
+      <c r="AD8" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE8" s="8">
+        <v>30610</v>
+      </c>
+      <c r="AF8" s="7">
+        <v>427800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32">
       <c r="A9" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B9" s="12">
         <v>0.2</v>
@@ -1994,26 +2080,26 @@
         <v>65000</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J9" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
+        <f>SUM(Inputs!$B$28:$C$28)+AE9</f>
         <v>109290</v>
       </c>
       <c r="K9" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
+        <f>SUM(Inputs!$B$29:$C$29)+AF9</f>
         <v>1915828.04</v>
       </c>
       <c r="L9" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE9/Inputs!$D$28</f>
         <v>216051.47</v>
       </c>
       <c r="M9" s="11">
-        <f>Inputs!$B$29*(B9+C9)/2+Inputs!$C$29*(D9+E9)/2+Inputs!$D$29*(F9+G9)/2</f>
+        <f>Inputs!$B$29*(B9+C9)/2+Inputs!$C$29*(D9+E9)/2+AF9*(F9+G9)/2</f>
         <v>293682.9672</v>
       </c>
       <c r="N9" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE9/Inputs!$D$28</f>
         <v>363478.82355999993</v>
       </c>
       <c r="O9" s="10">
@@ -2025,7 +2111,7 @@
         <v>0.07634067911439489</v>
       </c>
       <c r="Q9" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE9/Inputs!$D$28</f>
         <v>129749.6</v>
       </c>
       <c r="R9" s="15">
@@ -2041,11 +2127,11 @@
         <v>0.008615602911835505</v>
       </c>
       <c r="U9" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(AE9=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="V9" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
+        <f>Inputs!$B$9+IF(AE9=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>25415.45</v>
       </c>
       <c r="W9" s="15">
@@ -2068,10 +2154,27 @@
         <f>$M$6-M9</f>
         <v>42190.52279999998</v>
       </c>
-    </row>
-    <row r="10" spans="1:27">
+      <c r="AB9" s="11">
+        <f>L9/J9</f>
+        <v>1.9768640314758898</v>
+      </c>
+      <c r="AC9" s="13">
+        <f>L9/K9</f>
+        <v>0.1127718487719806</v>
+      </c>
+      <c r="AD9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE9" s="8">
+        <v>50400</v>
+      </c>
+      <c r="AF9" s="7">
+        <v>852768</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32">
       <c r="A10" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B10" s="12">
         <v>0.16</v>
@@ -2095,26 +2198,26 @@
         <v>65000</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="J10" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
+        <f>SUM(Inputs!$B$28:$C$28)+AE10</f>
         <v>109290</v>
       </c>
       <c r="K10" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
+        <f>SUM(Inputs!$B$29:$C$29)+AF10</f>
         <v>1915828.04</v>
       </c>
       <c r="L10" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE10/Inputs!$D$28</f>
         <v>216051.47</v>
       </c>
       <c r="M10" s="11">
-        <f>Inputs!$B$29*(B10+C10)/2+Inputs!$C$29*(D10+E10)/2+Inputs!$D$29*(F10+G10)/2</f>
+        <f>Inputs!$B$29*(B10+C10)/2+Inputs!$C$29*(D10+E10)/2+AF10*(F10+G10)/2</f>
         <v>272421.76639999996</v>
       </c>
       <c r="N10" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE10/Inputs!$D$28</f>
         <v>363478.82355999993</v>
       </c>
       <c r="O10" s="10">
@@ -2126,7 +2229,7 @@
         <v>0.06524302298028795</v>
       </c>
       <c r="Q10" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE10/Inputs!$D$28</f>
         <v>129749.6</v>
       </c>
       <c r="R10" s="15">
@@ -2142,11 +2245,11 @@
         <v>-0.0024820532222714527</v>
       </c>
       <c r="U10" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(AE10=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="V10" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
+        <f>Inputs!$B$9+IF(AE10=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>25415.45</v>
       </c>
       <c r="W10" s="15">
@@ -2169,10 +2272,27 @@
         <f>$M$6-M10</f>
         <v>63451.72360000003</v>
       </c>
-    </row>
-    <row r="11" spans="1:27">
+      <c r="AB10" s="11">
+        <f>L10/J10</f>
+        <v>1.9768640314758898</v>
+      </c>
+      <c r="AC10" s="13">
+        <f>L10/K10</f>
+        <v>0.1127718487719806</v>
+      </c>
+      <c r="AD10" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE10" s="8">
+        <v>50400</v>
+      </c>
+      <c r="AF10" s="7">
+        <v>852768</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32">
       <c r="A11" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B11" s="12">
         <v>0.2</v>
@@ -2196,26 +2316,26 @@
         <v>65000</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="J11" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
+        <f>SUM(Inputs!$B$28:$C$28)+AE11</f>
         <v>109290</v>
       </c>
       <c r="K11" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
+        <f>SUM(Inputs!$B$29:$C$29)+AF11</f>
         <v>1915828.04</v>
       </c>
       <c r="L11" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE11/Inputs!$D$28</f>
         <v>216051.47</v>
       </c>
       <c r="M11" s="11">
-        <f>Inputs!$B$29*(B11+C11)/2+Inputs!$C$29*(D11+E11)/2+Inputs!$D$29*(F11+G11)/2</f>
+        <f>Inputs!$B$29*(B11+C11)/2+Inputs!$C$29*(D11+E11)/2+AF11*(F11+G11)/2</f>
         <v>310738.32720000006</v>
       </c>
       <c r="N11" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE11/Inputs!$D$28</f>
         <v>363478.82355999993</v>
       </c>
       <c r="O11" s="10">
@@ -2227,7 +2347,7 @@
         <v>0.08524302298028799</v>
       </c>
       <c r="Q11" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE11/Inputs!$D$28</f>
         <v>129749.6</v>
       </c>
       <c r="R11" s="15">
@@ -2243,11 +2363,11 @@
         <v>0.017517946777728596</v>
       </c>
       <c r="U11" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(AE11=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="V11" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
+        <f>Inputs!$B$9+IF(AE11=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>25415.45</v>
       </c>
       <c r="W11" s="15">
@@ -2270,10 +2390,27 @@
         <f>$M$6-M11</f>
         <v>25135.162799999933</v>
       </c>
-    </row>
-    <row r="12" spans="1:27">
+      <c r="AB11" s="11">
+        <f>L11/J11</f>
+        <v>1.9768640314758898</v>
+      </c>
+      <c r="AC11" s="13">
+        <f>L11/K11</f>
+        <v>0.1127718487719806</v>
+      </c>
+      <c r="AD11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE11" s="8">
+        <v>50400</v>
+      </c>
+      <c r="AF11" s="7">
+        <v>852768</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32">
       <c r="A12" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B12" s="12">
         <v>0.16</v>
@@ -2297,26 +2434,26 @@
         <v>65000</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="J12" s="9">
-        <f>SUM(Inputs!$B$28:$D$28)</f>
+        <f>SUM(Inputs!$B$28:$C$28)+AE12</f>
         <v>109290</v>
       </c>
       <c r="K12" s="11">
-        <f>SUM(Inputs!$B$29:$D$29)</f>
+        <f>SUM(Inputs!$B$29:$C$29)+AF12</f>
         <v>1915828.04</v>
       </c>
       <c r="L12" s="11">
-        <f>SUM(Inputs!$B$30:$D$30)</f>
+        <f>SUM(Inputs!$B$30:$C$30)+Inputs!$D$30*AE12/Inputs!$D$28</f>
         <v>216051.47</v>
       </c>
       <c r="M12" s="11">
-        <f>Inputs!$B$29*(B12+C12)/2+Inputs!$C$29*(D12+E12)/2+Inputs!$D$29*(F12+G12)/2</f>
+        <f>Inputs!$B$29*(B12+C12)/2+Inputs!$C$29*(D12+E12)/2+AF12*(F12+G12)/2</f>
         <v>306532.4864</v>
       </c>
       <c r="N12" s="11">
-        <f>SUM(Inputs!$B$31:$D$31)</f>
+        <f>SUM(Inputs!$B$31:$C$31)+Inputs!$D$31*AE12/Inputs!$D$28</f>
         <v>363478.82355999993</v>
       </c>
       <c r="O12" s="10">
@@ -2328,7 +2465,7 @@
         <v>0.08304771071207419</v>
       </c>
       <c r="Q12" s="11">
-        <f>SUM(Inputs!$B$32:$D$32)</f>
+        <f>SUM(Inputs!$B$32:$C$32)+Inputs!$D$32*AE12/Inputs!$D$28</f>
         <v>129749.6</v>
       </c>
       <c r="R12" s="15">
@@ -2344,11 +2481,11 @@
         <v>0.015322634509514793</v>
       </c>
       <c r="U12" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(AE12=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="V12" s="15">
-        <f>Inputs!$B$9+Inputs!$B$10</f>
+        <f>Inputs!$B$9+IF(AE12=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>25415.45</v>
       </c>
       <c r="W12" s="15">
@@ -2371,9 +2508,26 @@
         <f>$M$6-M12</f>
         <v>29341.003599999996</v>
       </c>
+      <c r="AB12" s="11">
+        <f>L12/J12</f>
+        <v>1.9768640314758898</v>
+      </c>
+      <c r="AC12" s="13">
+        <f>L12/K12</f>
+        <v>0.1127718487719806</v>
+      </c>
+      <c r="AD12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE12" s="8">
+        <v>50400</v>
+      </c>
+      <c r="AF12" s="7">
+        <v>852768</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:AA12"/>
+  <autoFilter ref="A5:AF12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A3:Z3"/>
@@ -2393,7 +2547,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2417,7 +2571,7 @@
     </row>
     <row r="3" spans="1:21">
       <c r="A3" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2444,7 +2598,7 @@
         <v>54</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>63</v>
@@ -2453,16 +2607,16 @@
         <v>64</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>65</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>66</v>
@@ -2480,7 +2634,7 @@
         <v>70</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>72</v>
@@ -2506,10 +2660,10 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C6" s="9">
         <f>Inputs!$B$28</f>
@@ -2524,7 +2678,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F6" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C6/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G6" s="13">
@@ -2540,7 +2694,7 @@
         <v>207245.02</v>
       </c>
       <c r="J6" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C6/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K6" s="10">
@@ -2552,7 +2706,7 @@
         <v>0.1332644596274894</v>
       </c>
       <c r="M6" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C6/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N6" s="15">
@@ -2590,7 +2744,7 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>32</v>
@@ -2608,7 +2762,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F7" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C7/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G7" s="13">
@@ -2624,7 +2778,7 @@
         <v>7668.47</v>
       </c>
       <c r="J7" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C7/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K7" s="10">
@@ -2636,7 +2790,7 @@
         <v>0.14641882662920097</v>
       </c>
       <c r="M7" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C7/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N7" s="15">
@@ -2674,25 +2828,25 @@
     </row>
     <row r="8" spans="1:21">
       <c r="A8" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="9">
-        <f>Inputs!$D$28</f>
+        <f>Scenarios!$AE$6</f>
         <v>50400</v>
       </c>
       <c r="D8" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$6</f>
+        <v>852768</v>
       </c>
       <c r="E8" s="11">
         <f>D8/C8</f>
         <v>16.92</v>
       </c>
       <c r="F8" s="11">
-        <f>Inputs!$D$30</f>
+        <f>Inputs!$D$30*C8/Inputs!$D$28</f>
         <v>96768.0</v>
       </c>
       <c r="G8" s="13">
@@ -2708,7 +2862,7 @@
         <v>136442.88</v>
       </c>
       <c r="J8" s="11">
-        <f>Inputs!$D$31</f>
+        <f>Inputs!$D$31*C8/Inputs!$D$28</f>
         <v>171397.71356</v>
       </c>
       <c r="K8" s="10">
@@ -2720,7 +2874,7 @@
         <v>0.07248532595031709</v>
       </c>
       <c r="M8" s="11">
-        <f>Inputs!$D$32</f>
+        <f>Inputs!$D$32*C8/Inputs!$D$28</f>
         <v>28728.0</v>
       </c>
       <c r="N8" s="15">
@@ -2736,11 +2890,11 @@
         <v>0.03879738268790574</v>
       </c>
       <c r="Q8" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(C8=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="R8" s="15">
-        <f>Inputs!$B$10</f>
+        <f>IF(C8=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>10800</v>
       </c>
       <c r="S8" s="15">
@@ -2758,10 +2912,10 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C10" s="9">
         <f>Inputs!$B$28</f>
@@ -2776,7 +2930,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F10" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C10/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G10" s="13">
@@ -2792,7 +2946,7 @@
         <v>257255.8925</v>
       </c>
       <c r="J10" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C10/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K10" s="10">
@@ -2804,7 +2958,7 @@
         <v>0.1818647774025235</v>
       </c>
       <c r="M10" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C10/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N10" s="15">
@@ -2829,20 +2983,20 @@
       </c>
       <c r="S10" s="15">
         <f>Inputs!$B$11*D10/SUM(Inputs!$B$29:$D$29)</f>
-        <v>5371.168750615008</v>
+        <v>6902.214442611259</v>
       </c>
       <c r="T10" s="10">
         <f>O10-Q10-R10-S10</f>
-        <v>68604.76316592176</v>
+        <v>67073.7174739255</v>
       </c>
       <c r="U10" s="13">
         <f>T10/D10</f>
-        <v>0.06666976847374037</v>
+        <v>0.06518190586628206</v>
       </c>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>32</v>
@@ -2860,7 +3014,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F11" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C11/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G11" s="13">
@@ -2876,7 +3030,7 @@
         <v>8509.1175</v>
       </c>
       <c r="J11" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C11/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K11" s="10">
@@ -2888,7 +3042,7 @@
         <v>0.17111726039745012</v>
       </c>
       <c r="M11" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C11/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N11" s="15">
@@ -2913,39 +3067,39 @@
       </c>
       <c r="S11" s="15">
         <f>Inputs!$B$11*D11/SUM(Inputs!$B$29:$D$29)</f>
-        <v>177.65931643844195</v>
+        <v>228.30090744131823</v>
       </c>
       <c r="T11" s="10">
         <f>O11-Q11-R11-S11</f>
-        <v>3176.728767024839</v>
+        <v>3126.087176021963</v>
       </c>
       <c r="U11" s="13">
         <f>T11/D11</f>
-        <v>0.09333308557041428</v>
+        <v>0.091845222962956</v>
       </c>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="9">
-        <f>Inputs!$D$28</f>
-        <v>50400</v>
+        <f>Scenarios!$AE$7</f>
+        <v>30610</v>
       </c>
       <c r="D12" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$7</f>
+        <v>427800</v>
       </c>
       <c r="E12" s="11">
         <f>D12/C12</f>
-        <v>16.92</v>
+        <v>13.975824893825548</v>
       </c>
       <c r="F12" s="11">
-        <f>Inputs!$D$30</f>
-        <v>96768.0</v>
+        <f>Inputs!$D$30*C12/Inputs!$D$28</f>
+        <v>58771.2</v>
       </c>
       <c r="G12" s="13">
         <f>Scenarios!$F$7</f>
@@ -2957,23 +3111,23 @@
       </c>
       <c r="I12" s="11">
         <f>D12*(G12+H12)/2</f>
-        <v>102332.15999999999</v>
+        <v>51336.0</v>
       </c>
       <c r="J12" s="11">
-        <f>Inputs!$D$31</f>
-        <v>171397.71356</v>
+        <f>Inputs!$D$31*C12/Inputs!$D$28</f>
+        <v>104096.90500142063</v>
       </c>
       <c r="K12" s="10">
         <f>I12+F12-J12</f>
-        <v>27702.44643999997</v>
+        <v>6010.2949985793675</v>
       </c>
       <c r="L12" s="13">
         <f>K12/D12</f>
-        <v>0.03248532595031705</v>
+        <v>0.007047983740688402</v>
       </c>
       <c r="M12" s="11">
-        <f>Inputs!$D$32</f>
-        <v>28728.0</v>
+        <f>Inputs!$D$32*C12/Inputs!$D$28</f>
+        <v>17447.699999999997</v>
       </c>
       <c r="N12" s="15">
         <f>0</f>
@@ -2981,39 +3135,39 @@
       </c>
       <c r="O12" s="10">
         <f>K12-M12</f>
-        <v>-1025.5535600000294</v>
+        <v>-11437.40500142063</v>
       </c>
       <c r="P12" s="13">
         <f>O12/D12</f>
-        <v>-0.0012026173120942968</v>
+        <v>-0.013412094498645152</v>
       </c>
       <c r="Q12" s="15">
-        <f>Inputs!$B$7</f>
-        <v>28000</v>
+        <f>IF(C12=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
+        <v>14000</v>
       </c>
       <c r="R12" s="15">
-        <f>Inputs!$B$10</f>
-        <v>10800</v>
+        <f>IF(C12=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
+        <v>5400</v>
       </c>
       <c r="S12" s="15">
         <f>Inputs!$B$11*D12/SUM(Inputs!$B$29:$D$29)</f>
-        <v>4451.1719329465495</v>
+        <v>2869.4846499474224</v>
       </c>
       <c r="T12" s="16">
         <f>O12-Q12-R12-S12</f>
-        <v>-44276.72549294658</v>
+        <v>-33706.88965136805</v>
       </c>
       <c r="U12" s="13">
         <f>T12/D12</f>
-        <v>-0.05192118547242225</v>
+        <v>-0.039526447581719824</v>
       </c>
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C14" s="9">
         <f>Inputs!$B$28</f>
@@ -3028,7 +3182,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F14" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C14/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G14" s="13">
@@ -3044,7 +3198,7 @@
         <v>231530.30325</v>
       </c>
       <c r="J14" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C14/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K14" s="10">
@@ -3056,7 +3210,7 @@
         <v>0.15686477740252347</v>
       </c>
       <c r="M14" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C14/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N14" s="15">
@@ -3081,20 +3235,20 @@
       </c>
       <c r="S14" s="15">
         <f>Inputs!$B$11*D14/SUM(Inputs!$B$29:$D$29)</f>
-        <v>5371.168750615008</v>
+        <v>6902.214442611259</v>
       </c>
       <c r="T14" s="10">
         <f>O14-Q14-R14-S14</f>
-        <v>42879.173915921725</v>
+        <v>41348.12822392548</v>
       </c>
       <c r="U14" s="13">
         <f>T14/D14</f>
-        <v>0.041669768473740335</v>
+        <v>0.040181905866282036</v>
       </c>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>32</v>
@@ -3112,7 +3266,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F15" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C15/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G15" s="13">
@@ -3128,7 +3282,7 @@
         <v>7658.20575</v>
       </c>
       <c r="J15" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C15/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K15" s="10">
@@ -3140,7 +3294,7 @@
         <v>0.14611726039745013</v>
       </c>
       <c r="M15" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C15/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N15" s="15">
@@ -3165,39 +3319,39 @@
       </c>
       <c r="S15" s="15">
         <f>Inputs!$B$11*D15/SUM(Inputs!$B$29:$D$29)</f>
-        <v>177.65931643844195</v>
+        <v>228.30090744131823</v>
       </c>
       <c r="T15" s="10">
         <f>O15-Q15-R15-S15</f>
-        <v>2325.8170170248395</v>
+        <v>2275.1754260219636</v>
       </c>
       <c r="U15" s="13">
         <f>T15/D15</f>
-        <v>0.0683330855704143</v>
+        <v>0.06684522296295602</v>
       </c>
     </row>
     <row r="16" spans="1:21">
       <c r="A16" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="9">
-        <f>Inputs!$D$28</f>
-        <v>50400</v>
+        <f>Scenarios!$AE$8</f>
+        <v>30610</v>
       </c>
       <c r="D16" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$8</f>
+        <v>427800</v>
       </c>
       <c r="E16" s="11">
         <f>D16/C16</f>
-        <v>16.92</v>
+        <v>13.975824893825548</v>
       </c>
       <c r="F16" s="11">
-        <f>Inputs!$D$30</f>
-        <v>96768.0</v>
+        <f>Inputs!$D$30*C16/Inputs!$D$28</f>
+        <v>58771.2</v>
       </c>
       <c r="G16" s="13">
         <f>Scenarios!$F$8</f>
@@ -3209,23 +3363,23 @@
       </c>
       <c r="I16" s="11">
         <f>D16*(G16+H16)/2</f>
-        <v>102332.15999999999</v>
+        <v>51336.0</v>
       </c>
       <c r="J16" s="11">
-        <f>Inputs!$D$31</f>
-        <v>171397.71356</v>
+        <f>Inputs!$D$31*C16/Inputs!$D$28</f>
+        <v>104096.90500142063</v>
       </c>
       <c r="K16" s="10">
         <f>I16+F16-J16</f>
-        <v>27702.44643999997</v>
+        <v>6010.2949985793675</v>
       </c>
       <c r="L16" s="13">
         <f>K16/D16</f>
-        <v>0.03248532595031705</v>
+        <v>0.007047983740688402</v>
       </c>
       <c r="M16" s="11">
-        <f>Inputs!$D$32</f>
-        <v>28728.0</v>
+        <f>Inputs!$D$32*C16/Inputs!$D$28</f>
+        <v>17447.699999999997</v>
       </c>
       <c r="N16" s="15">
         <f>0</f>
@@ -3233,39 +3387,39 @@
       </c>
       <c r="O16" s="10">
         <f>K16-M16</f>
-        <v>-1025.5535600000294</v>
+        <v>-11437.40500142063</v>
       </c>
       <c r="P16" s="13">
         <f>O16/D16</f>
-        <v>-0.0012026173120942968</v>
+        <v>-0.013412094498645152</v>
       </c>
       <c r="Q16" s="15">
-        <f>Inputs!$B$7</f>
-        <v>28000</v>
+        <f>IF(C16=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
+        <v>14000</v>
       </c>
       <c r="R16" s="15">
-        <f>Inputs!$B$10</f>
-        <v>10800</v>
+        <f>IF(C16=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
+        <v>5400</v>
       </c>
       <c r="S16" s="15">
         <f>Inputs!$B$11*D16/SUM(Inputs!$B$29:$D$29)</f>
-        <v>4451.1719329465495</v>
+        <v>2869.4846499474224</v>
       </c>
       <c r="T16" s="16">
         <f>O16-Q16-R16-S16</f>
-        <v>-44276.72549294658</v>
+        <v>-33706.88965136805</v>
       </c>
       <c r="U16" s="13">
         <f>T16/D16</f>
-        <v>-0.05192118547242225</v>
+        <v>-0.039526447581719824</v>
       </c>
     </row>
     <row r="18" spans="1:21">
       <c r="A18" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C18" s="9">
         <f>Inputs!$B$28</f>
@@ -3280,7 +3434,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F18" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C18/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G18" s="13">
@@ -3296,7 +3450,7 @@
         <v>185224.2426</v>
       </c>
       <c r="J18" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C18/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K18" s="10">
@@ -3308,7 +3462,7 @@
         <v>0.11186477740252347</v>
       </c>
       <c r="M18" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C18/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N18" s="15">
@@ -3346,7 +3500,7 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>32</v>
@@ -3364,7 +3518,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F19" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C19/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G19" s="13">
@@ -3380,7 +3534,7 @@
         <v>6126.5646</v>
       </c>
       <c r="J19" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C19/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K19" s="10">
@@ -3392,7 +3546,7 @@
         <v>0.1011172603974501</v>
       </c>
       <c r="M19" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C19/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N19" s="15">
@@ -3430,25 +3584,25 @@
     </row>
     <row r="20" spans="1:21">
       <c r="A20" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="9">
-        <f>Inputs!$D$28</f>
+        <f>Scenarios!$AE$9</f>
         <v>50400</v>
       </c>
       <c r="D20" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$9</f>
+        <v>852768</v>
       </c>
       <c r="E20" s="11">
         <f>D20/C20</f>
         <v>16.92</v>
       </c>
       <c r="F20" s="11">
-        <f>Inputs!$D$30</f>
+        <f>Inputs!$D$30*C20/Inputs!$D$28</f>
         <v>96768.0</v>
       </c>
       <c r="G20" s="13">
@@ -3464,7 +3618,7 @@
         <v>102332.15999999999</v>
       </c>
       <c r="J20" s="11">
-        <f>Inputs!$D$31</f>
+        <f>Inputs!$D$31*C20/Inputs!$D$28</f>
         <v>171397.71356</v>
       </c>
       <c r="K20" s="10">
@@ -3476,7 +3630,7 @@
         <v>0.03248532595031705</v>
       </c>
       <c r="M20" s="11">
-        <f>Inputs!$D$32</f>
+        <f>Inputs!$D$32*C20/Inputs!$D$28</f>
         <v>28728.0</v>
       </c>
       <c r="N20" s="15">
@@ -3492,11 +3646,11 @@
         <v>-0.0012026173120942968</v>
       </c>
       <c r="Q20" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(C20=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="R20" s="15">
-        <f>Inputs!$B$10</f>
+        <f>IF(C20=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>10800</v>
       </c>
       <c r="S20" s="15">
@@ -3514,10 +3668,10 @@
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C22" s="9">
         <f>Inputs!$B$28</f>
@@ -3532,7 +3686,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F22" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C22/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G22" s="13">
@@ -3548,7 +3702,7 @@
         <v>164643.7712</v>
       </c>
       <c r="J22" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C22/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K22" s="10">
@@ -3560,7 +3714,7 @@
         <v>0.0918647774025235</v>
       </c>
       <c r="M22" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C22/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N22" s="15">
@@ -3598,7 +3752,7 @@
     </row>
     <row r="23" spans="1:21">
       <c r="A23" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>32</v>
@@ -3616,7 +3770,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F23" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C23/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G23" s="13">
@@ -3632,7 +3786,7 @@
         <v>5445.8352</v>
       </c>
       <c r="J23" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C23/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K23" s="10">
@@ -3644,7 +3798,7 @@
         <v>0.08111726039745015</v>
       </c>
       <c r="M23" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C23/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N23" s="15">
@@ -3682,25 +3836,25 @@
     </row>
     <row r="24" spans="1:21">
       <c r="A24" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C24" s="9">
-        <f>Inputs!$D$28</f>
+        <f>Scenarios!$AE$10</f>
         <v>50400</v>
       </c>
       <c r="D24" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$10</f>
+        <v>852768</v>
       </c>
       <c r="E24" s="11">
         <f>D24/C24</f>
         <v>16.92</v>
       </c>
       <c r="F24" s="11">
-        <f>Inputs!$D$30</f>
+        <f>Inputs!$D$30*C24/Inputs!$D$28</f>
         <v>96768.0</v>
       </c>
       <c r="G24" s="13">
@@ -3716,7 +3870,7 @@
         <v>102332.15999999999</v>
       </c>
       <c r="J24" s="11">
-        <f>Inputs!$D$31</f>
+        <f>Inputs!$D$31*C24/Inputs!$D$28</f>
         <v>171397.71356</v>
       </c>
       <c r="K24" s="10">
@@ -3728,7 +3882,7 @@
         <v>0.03248532595031705</v>
       </c>
       <c r="M24" s="11">
-        <f>Inputs!$D$32</f>
+        <f>Inputs!$D$32*C24/Inputs!$D$28</f>
         <v>28728.0</v>
       </c>
       <c r="N24" s="15">
@@ -3744,11 +3898,11 @@
         <v>-0.0012026173120942968</v>
       </c>
       <c r="Q24" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(C24=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="R24" s="15">
-        <f>Inputs!$B$10</f>
+        <f>IF(C24=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>10800</v>
       </c>
       <c r="S24" s="15">
@@ -3766,10 +3920,10 @@
     </row>
     <row r="26" spans="1:21">
       <c r="A26" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C26" s="9">
         <f>Inputs!$B$28</f>
@@ -3784,7 +3938,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F26" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C26/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G26" s="13">
@@ -3800,7 +3954,7 @@
         <v>185224.2426</v>
       </c>
       <c r="J26" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C26/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K26" s="10">
@@ -3812,7 +3966,7 @@
         <v>0.11186477740252347</v>
       </c>
       <c r="M26" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C26/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N26" s="15">
@@ -3850,7 +4004,7 @@
     </row>
     <row r="27" spans="1:21">
       <c r="A27" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>32</v>
@@ -3868,7 +4022,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F27" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C27/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G27" s="13">
@@ -3884,7 +4038,7 @@
         <v>6126.5646</v>
       </c>
       <c r="J27" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C27/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K27" s="10">
@@ -3896,7 +4050,7 @@
         <v>0.1011172603974501</v>
       </c>
       <c r="M27" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C27/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N27" s="15">
@@ -3934,25 +4088,25 @@
     </row>
     <row r="28" spans="1:21">
       <c r="A28" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C28" s="9">
-        <f>Inputs!$D$28</f>
+        <f>Scenarios!$AE$11</f>
         <v>50400</v>
       </c>
       <c r="D28" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$11</f>
+        <v>852768</v>
       </c>
       <c r="E28" s="11">
         <f>D28/C28</f>
         <v>16.92</v>
       </c>
       <c r="F28" s="11">
-        <f>Inputs!$D$30</f>
+        <f>Inputs!$D$30*C28/Inputs!$D$28</f>
         <v>96768.0</v>
       </c>
       <c r="G28" s="13">
@@ -3968,7 +4122,7 @@
         <v>119387.52000000002</v>
       </c>
       <c r="J28" s="11">
-        <f>Inputs!$D$31</f>
+        <f>Inputs!$D$31*C28/Inputs!$D$28</f>
         <v>171397.71356</v>
       </c>
       <c r="K28" s="10">
@@ -3980,7 +4134,7 @@
         <v>0.0524853259503171</v>
       </c>
       <c r="M28" s="11">
-        <f>Inputs!$D$32</f>
+        <f>Inputs!$D$32*C28/Inputs!$D$28</f>
         <v>28728.0</v>
       </c>
       <c r="N28" s="15">
@@ -3996,11 +4150,11 @@
         <v>0.018797382687905755</v>
       </c>
       <c r="Q28" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(C28=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="R28" s="15">
-        <f>Inputs!$B$10</f>
+        <f>IF(C28=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>10800</v>
       </c>
       <c r="S28" s="15">
@@ -4018,10 +4172,10 @@
     </row>
     <row r="30" spans="1:21">
       <c r="A30" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C30" s="9">
         <f>Inputs!$B$28</f>
@@ -4036,7 +4190,7 @@
         <v>18.066039958566687</v>
       </c>
       <c r="F30" s="11">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$30*C30/Inputs!$B$28</f>
         <v>115473.31</v>
       </c>
       <c r="G30" s="13">
@@ -4052,7 +4206,7 @@
         <v>164643.7712</v>
       </c>
       <c r="J30" s="11">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$31*C30/Inputs!$B$28</f>
         <v>185586.05999999997</v>
       </c>
       <c r="K30" s="10">
@@ -4064,7 +4218,7 @@
         <v>0.0918647774025235</v>
       </c>
       <c r="M30" s="11">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$32*C30/Inputs!$B$28</f>
         <v>99019.71</v>
       </c>
       <c r="N30" s="15">
@@ -4102,7 +4256,7 @@
     </row>
     <row r="31" spans="1:21">
       <c r="A31" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>32</v>
@@ -4120,7 +4274,7 @@
         <v>17.626343863283275</v>
       </c>
       <c r="F31" s="11">
-        <f>Inputs!$C$30</f>
+        <f>Inputs!$C$30*C31/Inputs!$C$28</f>
         <v>3810.16</v>
       </c>
       <c r="G31" s="13">
@@ -4136,7 +4290,7 @@
         <v>5445.8352</v>
       </c>
       <c r="J31" s="11">
-        <f>Inputs!$C$31</f>
+        <f>Inputs!$C$31*C31/Inputs!$C$28</f>
         <v>6495.050000000001</v>
       </c>
       <c r="K31" s="10">
@@ -4148,7 +4302,7 @@
         <v>0.08111726039745015</v>
       </c>
       <c r="M31" s="11">
-        <f>Inputs!$C$32</f>
+        <f>Inputs!$C$32*C31/Inputs!$C$28</f>
         <v>2001.89</v>
       </c>
       <c r="N31" s="15">
@@ -4186,25 +4340,25 @@
     </row>
     <row r="32" spans="1:21">
       <c r="A32" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C32" s="9">
-        <f>Inputs!$D$28</f>
+        <f>Scenarios!$AE$12</f>
         <v>50400</v>
       </c>
       <c r="D32" s="11">
-        <f>Inputs!$D$29</f>
-        <v>852768.0</v>
+        <f>Scenarios!$AF$12</f>
+        <v>852768</v>
       </c>
       <c r="E32" s="11">
         <f>D32/C32</f>
         <v>16.92</v>
       </c>
       <c r="F32" s="11">
-        <f>Inputs!$D$30</f>
+        <f>Inputs!$D$30*C32/Inputs!$D$28</f>
         <v>96768.0</v>
       </c>
       <c r="G32" s="13">
@@ -4220,7 +4374,7 @@
         <v>136442.88</v>
       </c>
       <c r="J32" s="11">
-        <f>Inputs!$D$31</f>
+        <f>Inputs!$D$31*C32/Inputs!$D$28</f>
         <v>171397.71356</v>
       </c>
       <c r="K32" s="10">
@@ -4232,7 +4386,7 @@
         <v>0.07248532595031709</v>
       </c>
       <c r="M32" s="11">
-        <f>Inputs!$D$32</f>
+        <f>Inputs!$D$32*C32/Inputs!$D$28</f>
         <v>28728.0</v>
       </c>
       <c r="N32" s="15">
@@ -4248,11 +4402,11 @@
         <v>0.03879738268790574</v>
       </c>
       <c r="Q32" s="15">
-        <f>Inputs!$B$7</f>
+        <f>IF(C32=30610,Inputs!$B$7/2,Inputs!$B$7)</f>
         <v>28000</v>
       </c>
       <c r="R32" s="15">
-        <f>Inputs!$B$10</f>
+        <f>IF(C32=30610,Inputs!$B$10/2,Inputs!$B$10)</f>
         <v>10800</v>
       </c>
       <c r="S32" s="15">
@@ -4293,7 +4447,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4303,10 +4457,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>11</v>
@@ -4315,50 +4469,50 @@
         <v>13</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -4366,59 +4520,59 @@
         <v>65</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4426,19 +4580,19 @@
         <v>75</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>